<commit_message>
updates on IPA dashboard
Add potential participants filter
</commit_message>
<xml_diff>
--- a/FTM Score Weights 2026.xlsx
+++ b/FTM Score Weights 2026.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="2" documentId="8_{CF541428-8520-40CB-95F4-A7221B036C63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1D5D8492-BCCD-094A-9B5E-87346AED50F6}"/>
   <bookViews>
-    <workbookView xWindow="-8160" yWindow="-21000" windowWidth="38400" windowHeight="21000" activeTab="1" xr2:uid="{E7A1A669-C0F1-41FB-94C3-6238C033C2EE}"/>
+    <workbookView xWindow="1440" yWindow="660" windowWidth="28800" windowHeight="18980" activeTab="1" xr2:uid="{E7A1A669-C0F1-41FB-94C3-6238C033C2EE}"/>
   </bookViews>
   <sheets>
     <sheet name="12mo-20yr Call List " sheetId="2" r:id="rId1"/>
@@ -611,6 +611,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -631,12 +637,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1162,19 +1162,19 @@
       <c r="G1" s="5"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="19" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A3" s="17"/>
+      <c r="A3" s="19"/>
       <c r="B3" t="s">
         <v>14</v>
       </c>
       <c r="C3">
         <v>0</v>
       </c>
-      <c r="D3" s="22" t="s">
+      <c r="D3" s="24" t="s">
         <v>27</v>
       </c>
       <c r="E3" t="s">
@@ -1182,14 +1182,14 @@
       </c>
     </row>
     <row r="4" spans="1:7" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="18"/>
+      <c r="A4" s="20"/>
       <c r="B4" s="1" t="s">
         <v>15</v>
       </c>
       <c r="C4" s="1">
         <v>1</v>
       </c>
-      <c r="D4" s="23"/>
+      <c r="D4" s="25"/>
       <c r="E4" s="1" t="s">
         <v>1</v>
       </c>
@@ -1204,14 +1204,14 @@
       <c r="E5" s="2"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A6" s="22"/>
+      <c r="A6" s="24"/>
       <c r="B6" t="s">
         <v>14</v>
       </c>
       <c r="C6">
         <v>0</v>
       </c>
-      <c r="D6" s="22" t="s">
+      <c r="D6" s="24" t="s">
         <v>27</v>
       </c>
       <c r="E6" t="s">
@@ -1219,20 +1219,20 @@
       </c>
     </row>
     <row r="7" spans="1:7" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="23"/>
+      <c r="A7" s="25"/>
       <c r="B7" s="1" t="s">
         <v>15</v>
       </c>
       <c r="C7" s="1">
         <v>1</v>
       </c>
-      <c r="D7" s="23"/>
+      <c r="D7" s="25"/>
       <c r="E7" s="1" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A8" s="25" t="s">
+      <c r="A8" s="18" t="s">
         <v>17</v>
       </c>
       <c r="B8" s="2"/>
@@ -1241,14 +1241,14 @@
       <c r="E8" s="2"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A9" s="17"/>
+      <c r="A9" s="19"/>
       <c r="B9" t="s">
         <v>14</v>
       </c>
       <c r="C9">
         <v>0</v>
       </c>
-      <c r="D9" s="17" t="s">
+      <c r="D9" s="19" t="s">
         <v>24</v>
       </c>
       <c r="E9" t="s">
@@ -1256,20 +1256,20 @@
       </c>
     </row>
     <row r="10" spans="1:7" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="18"/>
+      <c r="A10" s="20"/>
       <c r="B10" s="1" t="s">
         <v>15</v>
       </c>
       <c r="C10" s="1">
         <v>1</v>
       </c>
-      <c r="D10" s="18"/>
+      <c r="D10" s="20"/>
       <c r="E10" s="1" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A11" s="25" t="s">
+      <c r="A11" s="18" t="s">
         <v>18</v>
       </c>
       <c r="B11" s="2"/>
@@ -1278,14 +1278,14 @@
       <c r="E11" s="2"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A12" s="17"/>
+      <c r="A12" s="19"/>
       <c r="B12" t="s">
         <v>14</v>
       </c>
       <c r="C12">
         <v>0</v>
       </c>
-      <c r="D12" s="17" t="s">
+      <c r="D12" s="19" t="s">
         <v>24</v>
       </c>
       <c r="E12" t="s">
@@ -1293,33 +1293,33 @@
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A13" s="17"/>
+      <c r="A13" s="19"/>
       <c r="B13" t="s">
         <v>15</v>
       </c>
       <c r="C13">
         <v>1</v>
       </c>
-      <c r="D13" s="17"/>
+      <c r="D13" s="19"/>
       <c r="E13" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="65" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="18"/>
+      <c r="A14" s="20"/>
       <c r="B14" s="1" t="s">
         <v>8</v>
       </c>
       <c r="C14" s="1">
         <v>1</v>
       </c>
-      <c r="D14" s="18"/>
+      <c r="D14" s="20"/>
       <c r="E14" s="4" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A15" s="25" t="s">
+      <c r="A15" s="18" t="s">
         <v>19</v>
       </c>
       <c r="B15" s="2"/>
@@ -1328,14 +1328,14 @@
       <c r="E15" s="2"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A16" s="17"/>
+      <c r="A16" s="19"/>
       <c r="B16" t="s">
         <v>20</v>
       </c>
       <c r="C16">
         <v>0</v>
       </c>
-      <c r="D16" s="17" t="s">
+      <c r="D16" s="19" t="s">
         <v>24</v>
       </c>
       <c r="E16" t="s">
@@ -1343,14 +1343,14 @@
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A17" s="17"/>
+      <c r="A17" s="19"/>
       <c r="B17" t="s">
         <v>21</v>
       </c>
       <c r="C17">
         <v>1</v>
       </c>
-      <c r="D17" s="17"/>
+      <c r="D17" s="19"/>
       <c r="E17" t="s">
         <v>9</v>
       </c>
@@ -1410,7 +1410,7 @@
       <c r="A2" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="B2" s="19">
+      <c r="B2" s="21">
         <v>2</v>
       </c>
       <c r="C2" s="7"/>
@@ -1419,15 +1419,15 @@
       <c r="F2" s="7"/>
     </row>
     <row r="3" spans="1:6" ht="48" x14ac:dyDescent="0.2">
-      <c r="A3" s="17"/>
-      <c r="B3" s="20"/>
+      <c r="A3" s="19"/>
+      <c r="B3" s="22"/>
       <c r="C3" t="s">
         <v>14</v>
       </c>
       <c r="D3">
         <v>0</v>
       </c>
-      <c r="E3" s="22" t="s">
+      <c r="E3" s="24" t="s">
         <v>31</v>
       </c>
       <c r="F3" s="8" t="s">
@@ -1435,29 +1435,29 @@
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A4" s="17"/>
-      <c r="B4" s="20"/>
+      <c r="A4" s="19"/>
+      <c r="B4" s="22"/>
       <c r="C4" t="s">
         <v>15</v>
       </c>
       <c r="D4">
         <v>1</v>
       </c>
-      <c r="E4" s="22"/>
+      <c r="E4" s="24"/>
       <c r="F4" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="18"/>
-      <c r="B5" s="21"/>
+      <c r="A5" s="20"/>
+      <c r="B5" s="23"/>
       <c r="C5" s="1" t="s">
         <v>30</v>
       </c>
       <c r="D5" s="1">
         <v>0.25</v>
       </c>
-      <c r="E5" s="23"/>
+      <c r="E5" s="25"/>
       <c r="F5" s="1" t="s">
         <v>33</v>
       </c>
@@ -1473,7 +1473,7 @@
       <c r="D6" s="2">
         <v>0</v>
       </c>
-      <c r="E6" s="25" t="s">
+      <c r="E6" s="18" t="s">
         <v>24</v>
       </c>
       <c r="F6" s="2" t="s">
@@ -1489,7 +1489,7 @@
       <c r="D7" s="9">
         <v>1</v>
       </c>
-      <c r="E7" s="24"/>
+      <c r="E7" s="17"/>
       <c r="F7" s="9" t="s">
         <v>49</v>
       </c>
@@ -1521,7 +1521,7 @@
       <c r="D9" s="9">
         <v>1</v>
       </c>
-      <c r="E9" s="24"/>
+      <c r="E9" s="17"/>
       <c r="F9" s="9" t="s">
         <v>50</v>
       </c>
@@ -1553,7 +1553,7 @@
       <c r="D11" s="9">
         <v>1</v>
       </c>
-      <c r="E11" s="24"/>
+      <c r="E11" s="17"/>
       <c r="F11" s="9" t="s">
         <v>51</v>
       </c>
@@ -1585,7 +1585,7 @@
       <c r="D13" s="9">
         <v>1</v>
       </c>
-      <c r="E13" s="24"/>
+      <c r="E13" s="17"/>
       <c r="F13" s="9" t="s">
         <v>44</v>
       </c>
@@ -1617,7 +1617,7 @@
       <c r="D15" s="9">
         <v>1</v>
       </c>
-      <c r="E15" s="24"/>
+      <c r="E15" s="17"/>
       <c r="F15" s="9" t="s">
         <v>53</v>
       </c>
@@ -1649,7 +1649,7 @@
       <c r="D17" s="9">
         <v>1</v>
       </c>
-      <c r="E17" s="24"/>
+      <c r="E17" s="17"/>
       <c r="F17" s="9" t="s">
         <v>55</v>
       </c>
@@ -1681,7 +1681,7 @@
       <c r="D19" s="9">
         <v>1</v>
       </c>
-      <c r="E19" s="24"/>
+      <c r="E19" s="17"/>
       <c r="F19" s="9" t="s">
         <v>57</v>
       </c>
@@ -1713,7 +1713,7 @@
       <c r="D21" s="9">
         <v>1</v>
       </c>
-      <c r="E21" s="24"/>
+      <c r="E21" s="17"/>
       <c r="F21" s="9" t="s">
         <v>59</v>
       </c>
@@ -1745,7 +1745,7 @@
       <c r="D23" s="9">
         <v>1</v>
       </c>
-      <c r="E23" s="24"/>
+      <c r="E23" s="17"/>
       <c r="F23" s="9" t="s">
         <v>61</v>
       </c>
@@ -1777,13 +1777,18 @@
       <c r="D25" s="9">
         <v>1</v>
       </c>
-      <c r="E25" s="24"/>
+      <c r="E25" s="17"/>
       <c r="F25" s="9" t="s">
         <v>62</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="B2:B5"/>
+    <mergeCell ref="E3:E5"/>
+    <mergeCell ref="E18:E19"/>
+    <mergeCell ref="E20:E21"/>
     <mergeCell ref="E22:E23"/>
     <mergeCell ref="E24:E25"/>
     <mergeCell ref="E6:E7"/>
@@ -1792,11 +1797,6 @@
     <mergeCell ref="E14:E15"/>
     <mergeCell ref="E16:E17"/>
     <mergeCell ref="E8:E9"/>
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="B2:B5"/>
-    <mergeCell ref="E3:E5"/>
-    <mergeCell ref="E18:E19"/>
-    <mergeCell ref="E20:E21"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>